<commit_message>
docs(parking-lot): close #20 VeritaQC Phase 1 -> C25
TASK: VeritaQC Phase 1 shipped end-to-end (Phase 0 schema through 1D
monthly PDF + attestation + owner-override fix). Move item #20 from
OPEN to CLOSED as C25 with the full PR list and shipped-feature
summary. Regenerate xlsx mirror per the standing rule.

PLAN:
  1. Remove #20 from OPEN.
  2. Add C25 entry with all 8 PRs (#364-#371) and the per-phase
     summary.
  3. Re-run scripts/build_parking_lot_xlsx.py and commit both files.

Self-check:
  - Counts: OPEN 11 -> 10, CLOSED 24 -> 25. Confirmed by build script
    output.
  - C24 -> C25 numbering preserves the audit-trail sequence.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -670,83 +670,31 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Live QC engine (Levey-Jennings + Westgard)</t>
+          <t>CMS-116 application support + state licensing tracking</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Open. Scoping doc required per Section 8 Process Rules
-("Large tasks: present a build breakdown first, get approval, THEN
-build") before any code.</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>XL (6+ weeks; flagship-scale)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>A daily-use QC workflow: Levey-Jennings charts, Westgard
-multi-rule violation detection, control lot management, automated QC
-scheduling. Today VeritaAssure documents QC posture (sign-offs,
-records, retention); it does not run the QC. The COLA segment (small
-physician-office labs, urgent care, ER) lives in daily QC and will
-pick the tool that draws their L-J chart.</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Perplexity competitor analysis (myLabCompliance.io),
-2026-05-10. Operator forwarded the analysis; no decision yet.</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. Multi-week scoping + multi-month
-v1 build. Comparable in scale to VeritaResponse (#17).
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>CMS-116 application support + state licensing tracking</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Open. Small build relative to the other competitor-driven
 candidates. Useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor (myLabCompliance.io) has this; useful at lab startup and...</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>CMS-116 is the federal CLIA application form. Today
 VeritaPolicy covers ongoing CLIA posture but not the application
@@ -756,13 +704,13 @@
 CLIA.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io),
 2026-05-10. myLabCompliance.io has this; VeritaAssure does not.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. ~1-2 weeks for v1 (CMS-116 form +
 top-10-state licensure registry).
@@ -770,33 +718,33 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Acquire CAP MOL (Molecular) checklist to verify 2 pending entries</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Open, blocks on operator obtaining the MOL checklist.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>N/A (operator action — ~1 hour of code work once the file is in hand)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Low — two entries total; low traffic; only matters when a customer cites a MO...</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>PR #108 left 2 entries in server/capRequirements.ts
 flagged as unverified because the operator does not hold the CAP MOL
@@ -810,48 +758,48 @@
 The MOL module's MAS xlsx is the only one missing from that set.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>PR #108 commit 92f9573 (closed via merge 2026-05-11),
 audit findings.</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. Two entries; low traffic.
 ---</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Acquire AABB Standards 35th edition + current COLA Accreditation Manual for exhaustive citation verification</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Open, blocks on operator obtaining the gated accreditor
 manuals. Until then, AABB / COLA citations are best-effort against
 the public-source compilations.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>N/A (operator action — ~1-2 days of audit re-run once the manuals are held)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>High — gates #5 from reaching "exhaustively verified" status for AABB and COLA.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>The 2026-05-11 QC audit found that VeritaScan, cfrRequirements
 cross-refs, and colaRequirements.ts cite about 180 AABB and COLA codes
@@ -871,14 +819,14 @@
  does not enumerate fully.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 QC/QA audit, documented in
 OneDrive\Lab\Regulatory\aaa Truth Master Document\PROVENANCE.md
 "Audit-coverage limits" section.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. Operator-side action item, no code
 work pending until the source documents land.
@@ -886,34 +834,34 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>VeritaStock barcode scanning (full mobile scan flow)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Parked pending first paid commitment.
 ---</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>L (12 working days, ~3 weeks calendar)</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>High — strategic moat vs Unity Lab Services ($30K+/yr); presold as included o...</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>The remaining barcode-scanning build for VeritaStock, scoped
 during the 2026-05-20 Pfizer follow-up discussion. Order-now reorder
@@ -922,7 +870,7 @@
 Services-class inventory product.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>2026-05-20 Pfizer follow-up session, after the order-now
 reorder document shipped (PR #286). Strategic decision documented in
@@ -933,31 +881,31 @@
 barcode scanning waits on revenue...</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Plain-language summary layer for verbatim CFR citations</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>M (multi-day content authoring across 96 Master List rows if redesigned corre...</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Medium — director readability win; no customer urgency.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>server/cfrRequirements.ts carries verbatim eCFR text in
 the description field (PR #301 closed #26). The verbatim text is
@@ -966,8 +914,8 @@
 director read faster.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency. Operator
 has not yet authorized a redesign attempt as of 2026-05-21.
@@ -975,29 +923,29 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Lab leader community / forum (paid subscription idea)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>XL (ongoing operational commitment, not a build) as paid; S (a few days to sp...</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Low as paid product (SWOT verdict: don't build); Medium as free lead-funnel a...</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Operator-floated 2026-05-22: a vetted online forum for
 laboratory leaders (directors, managers, supervisors). Pricing as
@@ -1010,51 +958,51 @@
 lab-leader water cooler.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Active vs view-only seat split</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Open. Real product change, ~1 week of engineering when prioritized. Not blocking any current customer; activate when a prospect explicitly asks "do you charge for our medical director?"</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>M (~1 week of engineering when prioritized)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Medium — quality-of-life for sales positioning; /pricing copy already claims...</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>The pricing analysis doc (2026-05-21 MEDIUM scenario, Decision 3) proposed splitting seats into two types: active (techs, supervisors, lab managers who edit data; counted against the tier seat cap) and view-only (medical director, administrators, reviewers who sign but don't enter; unlimited and free on every tier). The current schema treats all seats as one bucket.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Pricing analysis doc Decision 3 (2026-05-21); deferred during Phase B Stripe wiring (2026-05-23) because no current customer is constrained by the missing distinction.</t>
+        </is>
+      </c>
       <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Active vs view-only seat split</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Open. Real product change, ~1 week of engineering when prioritized. Not blocking any current customer; activate when a prospect explicitly asks "do you charge for our medical director?"</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>M (~1 week of engineering when prioritized)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Medium — quality-of-life for sales positioning; /pricing copy already claims...</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>The pricing analysis doc (2026-05-21 MEDIUM scenario, Decision 3) proposed splitting seats into two types: active (techs, supervisors, lab managers who edit data; counted against the tier seat cap) and view-only (medical director, administrators, reviewers who sign but don't enter; unlimited and free on every tier). The current schema treats all seats as one bucket.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pricing analysis doc Decision 3 (2026-05-21); deferred during Phase B Stripe wiring (2026-05-23) because no current customer is constrained by the missing distinction.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. Quality-of-life for sales positioning, not table stakes.
 ---
@@ -1064,7 +1012,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H12"/>
+  <autoFilter ref="A1:H11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1075,7 +1023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1916,8 +1864,44 @@
       </c>
       <c r="H25" s="3" t="inlineStr"/>
     </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
+Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
+---</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
+  <autoFilter ref="A1:H26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(parking-lot): close #20 VeritaQC Phase 1 -> C25 (#372)
TASK: VeritaQC Phase 1 shipped end-to-end (Phase 0 schema through 1D
monthly PDF + attestation + owner-override fix). Move item #20 from
OPEN to CLOSED as C25 with the full PR list and shipped-feature
summary. Regenerate xlsx mirror per the standing rule.

PLAN:
  1. Remove #20 from OPEN.
  2. Add C25 entry with all 8 PRs (#364-#371) and the per-phase
     summary.
  3. Re-run scripts/build_parking_lot_xlsx.py and commit both files.

Self-check:
  - Counts: OPEN 11 -> 10, CLOSED 24 -> 25. Confirmed by build script
    output.
  - C24 -> C25 numbering preserves the audit-trail sequence.

Co-authored-by: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -670,83 +670,31 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Live QC engine (Levey-Jennings + Westgard)</t>
+          <t>CMS-116 application support + state licensing tracking</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Open. Scoping doc required per Section 8 Process Rules
-("Large tasks: present a build breakdown first, get approval, THEN
-build") before any code.</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>XL (6+ weeks; flagship-scale)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>A daily-use QC workflow: Levey-Jennings charts, Westgard
-multi-rule violation detection, control lot management, automated QC
-scheduling. Today VeritaAssure documents QC posture (sign-offs,
-records, retention); it does not run the QC. The COLA segment (small
-physician-office labs, urgent care, ER) lives in daily QC and will
-pick the tool that draws their L-J chart.</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Perplexity competitor analysis (myLabCompliance.io),
-2026-05-10. Operator forwarded the analysis; no decision yet.</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. Multi-week scoping + multi-month
-v1 build. Comparable in scale to VeritaResponse (#17).
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>CMS-116 application support + state licensing tracking</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Open. Small build relative to the other competitor-driven
 candidates. Useful at lab startup and at certificate-type changes.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>M (1-2 weeks for v1)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Medium — competitor (myLabCompliance.io) has this; useful at lab startup and...</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>CMS-116 is the federal CLIA application form. Today
 VeritaPolicy covers ongoing CLIA posture but not the application
@@ -756,13 +704,13 @@
 CLIA.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io),
 2026-05-10. myLabCompliance.io has this; VeritaAssure does not.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. ~1-2 weeks for v1 (CMS-116 form +
 top-10-state licensure registry).
@@ -770,33 +718,33 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Acquire CAP MOL (Molecular) checklist to verify 2 pending entries</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Open, blocks on operator obtaining the MOL checklist.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>N/A (operator action — ~1 hour of code work once the file is in hand)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Low — two entries total; low traffic; only matters when a customer cites a MO...</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>PR #108 left 2 entries in server/capRequirements.ts
 flagged as unverified because the operator does not hold the CAP MOL
@@ -810,48 +758,48 @@
 The MOL module's MAS xlsx is the only one missing from that set.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>PR #108 commit 92f9573 (closed via merge 2026-05-11),
 audit findings.</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. Two entries; low traffic.
 ---</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Acquire AABB Standards 35th edition + current COLA Accreditation Manual for exhaustive citation verification</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Open, blocks on operator obtaining the gated accreditor
 manuals. Until then, AABB / COLA citations are best-effort against
 the public-source compilations.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>N/A (operator action — ~1-2 days of audit re-run once the manuals are held)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>High — gates #5 from reaching "exhaustively verified" status for AABB and COLA.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>The 2026-05-11 QC audit found that VeritaScan, cfrRequirements
 cross-refs, and colaRequirements.ts cite about 180 AABB and COLA codes
@@ -871,14 +819,14 @@
  does not enumerate fully.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>2026-05-11 QC/QA audit, documented in
 OneDrive\Lab\Regulatory\aaa Truth Master Document\PROVENANCE.md
 "Audit-coverage limits" section.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. Operator-side action item, no code
 work pending until the source documents land.
@@ -886,34 +834,34 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>VeritaStock barcode scanning (full mobile scan flow)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Parked pending first paid commitment.
 ---</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>L (12 working days, ~3 weeks calendar)</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>High — strategic moat vs Unity Lab Services ($30K+/yr); presold as included o...</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>The remaining barcode-scanning build for VeritaStock, scoped
 during the 2026-05-20 Pfizer follow-up discussion. Order-now reorder
@@ -922,7 +870,7 @@
 Services-class inventory product.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>2026-05-20 Pfizer follow-up session, after the order-now
 reorder document shipped (PR #286). Strategic decision documented in
@@ -933,31 +881,31 @@
 barcode scanning waits on revenue...</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Plain-language summary layer for verbatim CFR citations</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>M (multi-day content authoring across 96 Master List rows if redesigned corre...</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Medium — director readability win; no customer urgency.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>server/cfrRequirements.ts carries verbatim eCFR text in
 the description field (PR #301 closed #26). The verbatim text is
@@ -966,8 +914,8 @@
 director read faster.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Post-COLA. No customer urgency. Operator
 has not yet authorized a redesign attempt as of 2026-05-21.
@@ -975,29 +923,29 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Lab leader community / forum (paid subscription idea)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>XL (ongoing operational commitment, not a build) as paid; S (a few days to sp...</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Low as paid product (SWOT verdict: don't build); Medium as free lead-funnel a...</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Operator-floated 2026-05-22: a vetted online forum for
 laboratory leaders (directors, managers, supervisors). Pricing as
@@ -1010,51 +958,51 @@
 lab-leader water cooler.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Post-COLA. No customer urgency.
+---</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Active vs view-only seat split</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Open. Real product change, ~1 week of engineering when prioritized. Not blocking any current customer; activate when a prospect explicitly asks "do you charge for our medical director?"</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>M (~1 week of engineering when prioritized)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Medium — quality-of-life for sales positioning; /pricing copy already claims...</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>The pricing analysis doc (2026-05-21 MEDIUM scenario, Decision 3) proposed splitting seats into two types: active (techs, supervisors, lab managers who edit data; counted against the tier seat cap) and view-only (medical director, administrators, reviewers who sign but don't enter; unlimited and free on every tier). The current schema treats all seats as one bucket.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Pricing analysis doc Decision 3 (2026-05-21); deferred during Phase B Stripe wiring (2026-05-23) because no current customer is constrained by the missing distinction.</t>
+        </is>
+      </c>
       <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Post-COLA. No customer urgency.
----</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Active vs view-only seat split</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Open. Real product change, ~1 week of engineering when prioritized. Not blocking any current customer; activate when a prospect explicitly asks "do you charge for our medical director?"</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>M (~1 week of engineering when prioritized)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Medium — quality-of-life for sales positioning; /pricing copy already claims...</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>The pricing analysis doc (2026-05-21 MEDIUM scenario, Decision 3) proposed splitting seats into two types: active (techs, supervisors, lab managers who edit data; counted against the tier seat cap) and view-only (medical director, administrators, reviewers who sign but don't enter; unlimited and free on every tier). The current schema treats all seats as one bucket.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pricing analysis doc Decision 3 (2026-05-21); deferred during Phase B Stripe wiring (2026-05-23) because no current customer is constrained by the missing distinction.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Post-COLA. Quality-of-life for sales positioning, not table stakes.
 ---
@@ -1064,7 +1012,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H12"/>
+  <autoFilter ref="A1:H11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1075,7 +1023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1916,8 +1864,44 @@
       </c>
       <c r="H25" s="3" t="inlineStr"/>
     </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>VeritaQC Phase 1 (Levey-Jennings + Westgard live engine) (formerly #20)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B...</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>High — largest single gap vs myLabCompliance.io per Perplexity competitor ana...</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Effort: L (about 5 days end-to-end, actual: Phase 0 schema → Phase 1A evaluator → 1B entry UI → 1C daily review → 1D monthly PDF + attestation)
+Importance: High — largest single gap vs myLabCompliance.io per Perplexity competitor analysis; promotes VeritaAssure from documentation tool to lab operations platform.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Perplexity competitor analysis 2026-05-10. Scoping confirmed via the build_phase1_mockup.py iterations 2026-05-24. Shipped 2026-05-25.
+---</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
+  <autoFilter ref="A1:H26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(parking-lot): regenerate xlsx mirror for #22 rename
TASK: PR #373 committed PARKING_LOT.md alone because the xlsx was
locked. Regenerate now that the file is closed in Excel.

PLAN:
  1. Re-run scripts/build_parking_lot_xlsx.py.
  2. Stage + commit PARKING_LOT.xlsx onto the same branch.

Self-check:
  - Counts unchanged (10 OPEN / 25 CLOSED / 6 RETIRED).
  - Single-file commit on the same PR; no other drift.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -675,7 +675,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>CMS-116 application support + state licensing tracking</t>
+          <t>VeritaLab™ extension: CMS-116 application support + state licensing registry</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -696,18 +696,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>CMS-116 is the federal CLIA application form. Today
-VeritaPolicy covers ongoing CLIA posture but not the application
-itself. The form is also relevant at certificate-type changes (waived
-to moderate, moderate to high). State licensing tracking is the
-adjacent piece: many states require their own licensure on top of
-CLIA.</t>
+          <t>VeritaLab already tracks CLIA, state license, and lab
+director license as cert types in the certificate tracker. The
+missing pieces sit alongside that data:
+- CMS-116 form support: the federal CLIA application form. Lab
+ startup workflow and certificate-type changes (waived → moderate,
+ moderate → high) both require filing CMS-116. Today VeritaLab tracks
+ the resulting certificate but does not help author the application.
+- State licensure registry: many states require their own license
+ on top of CLIA. VeritaLab tracks the cert when held; the registry
+ piece is the per-state authority, form URL, fee, and renewal cadence
+ so the lab can look up the state-specific obligation.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Perplexity competitor analysis (myLabCompliance.io),
-2026-05-10. myLabCompliance.io has this; VeritaAssure does not.</t>
+2026-05-10. myLabCompliance.io has this; VeritaAssure does not.
+Reclassified as a VeritaLab extension 2026-05-25 (operator instinct:
+"it belongs with the VeritaLab module").</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore(parking-lot): close #33 — active vs view-only seat split shipped
TASK: Mark parking-lot #33 (active vs view-only seat split) as Done
2026-05-28. Six-PR sequence shipped today: #430-#435. PARKING_LOT.xlsx
mirror rebuilt to keep the Excel view in sync per memory rule.

PLAN:
  1. Update #33 Status line to Done with the PR list.
  2. Run scripts/build_parking_lot_xlsx.py to regenerate the mirror.
  3. Commit both files together.

Self-check:
  - Excel mirror drift? Re-ran builder; xlsx + md both reflect the
    same status text. Open count drops from 14 to 13.
  - STRIPE_VIEW_ONLY_ADDON_PRICE still unset — manual-invoice mode
    is the documented intent until the Stripe price is created.
  - Other open items untouched.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -986,7 +986,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Open. Foundation PR (step 1) ships in the session that locks the policy; steps 2-6 queue for a daylight multi-PR sprint.</t>
+          <t>Done 2026-05-28. Six-PR sequence shipped: #430 foundation (seat_type column, PLAN_VIEW_ONLY_SEATS scaffolding, admin report counts), #431 invite-flow seat_type, #432 dual-cap counting gates, #433 m...</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Post-COLA. Sales positioning gap; will close once the foundation ships.
+          <t>Post-COLA. Sales positioning gap; closed.
 ---
 _(items #34 and #35 closed 2026-05-24; see C23 and C24 below)_
 ---</t>

</xml_diff>

<commit_message>
chore(parking-lot): close #33 — active vs view-only seat split shipped (#436)
TASK: Mark parking-lot #33 (active vs view-only seat split) as Done
2026-05-28. Six-PR sequence shipped today: #430-#435. PARKING_LOT.xlsx
mirror rebuilt to keep the Excel view in sync per memory rule.

PLAN:
  1. Update #33 Status line to Done with the PR list.
  2. Run scripts/build_parking_lot_xlsx.py to regenerate the mirror.
  3. Commit both files together.

Self-check:
  - Excel mirror drift? Re-ran builder; xlsx + md both reflect the
    same status text. Open count drops from 14 to 13.
  - STRIPE_VIEW_ONLY_ADDON_PRICE still unset — manual-invoice mode
    is the documented intent until the Stripe price is created.
  - Other open items untouched.

Co-authored-by: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -986,7 +986,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Open. Foundation PR (step 1) ships in the session that locks the policy; steps 2-6 queue for a daylight multi-PR sprint.</t>
+          <t>Done 2026-05-28. Six-PR sequence shipped: #430 foundation (seat_type column, PLAN_VIEW_ONLY_SEATS scaffolding, admin report counts), #431 invite-flow seat_type, #432 dual-cap counting gates, #433 m...</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Post-COLA. Sales positioning gap; will close once the foundation ships.
+          <t>Post-COLA. Sales positioning gap; closed.
 ---
 _(items #34 and #35 closed 2026-05-24; see C23 and C24 below)_
 ---</t>

</xml_diff>

<commit_message>
chore(parking-lot): close C29 MediaLab functional mirror, add #39 parity hardening
TASK: Document the VeritaPolicy approval workflow build as Done (C29),
add #39 MediaLab parity hardening as open follow-on capturing the
60-70% surface assessment and the depth gaps surfaced by the QA pass.

PLAN:
  1. C29 entry: 12 PRs (#438-#449), schema + 8 phases + QA endpoint,
     54/54 happy-path verified.
  2. #39 entry: gaps list (quizzes, watermarking, SSO, delegation,
     etc.) with recommended sequence when customer-triggered.
  3. Re-run scripts/build_parking_lot_xlsx.py per memory rule.

Self-check:
  - Open count drops/rises correctly: was 10, now 11 (added #39).
  - Closed count rises: was 28, now 29 (added C29).
  - No accidental edits to other entries.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1005,8 +1005,56 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>MediaLab parity hardening (VeritaPolicy approval workflow depth)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Open, customer-triggered. No urgency until a prospect specifically asks for one of the listed depth items.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>L (1-2 weeks for the high-value items; each independent feature is M)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Medium-High — the C29 build shipped the surface MediaLab markets but depth is...</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>The VeritaPolicy approval workflow build (C29, 2026-05-29) hit roughly 60-70% MediaLab feature surface. The following gaps remain when comparing against an enterprise MediaLab Document Control deployment:
+- Quizzes on attestations. Schema columns quiz_score and quiz_total_questions exist on policy_attestations but the quiz authoring + presentation UI was scoped out of Phase 4. MediaLab labs use 5-10 multiple-choice questions per policy to confirm comprehension, not just attestation. Adds compliance defensibility.
+- PDF watermarking. MediaLab burns user name + timestamp into every downloaded PDF copy as a deterrent against forwarding. We serve clean originals. Add Puppeteer-style overlay at download time.
+- Per-policy role mapping at department level. MediaLab lets a lab say "only Microbiology Lab Director can approve Microbiology policies." Our required_role is per-step on the workflow, not per-document-by-manual.
+- Approval delegation. When a reviewer is on vacation, MediaLab supports temporary delegation to a designate. We have no delegation model.
+- In-browser DOCX editing. MediaLab has a structured editor that creates a Table of Contents from headings. We treat documents as...</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
+---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1017,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2002,8 +2050,44 @@
       </c>
       <c r="H29" s="3" t="inlineStr"/>
     </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>C29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>XL (one focused session, 12 PRs landed)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Effort: XL (one focused session, 12 PRs landed)
+Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
+---</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H29"/>
+  <autoFilter ref="A1:H30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(parking-lot): close C29 MediaLab functional mirror, add #39 parity hardening (#450)
TASK: Document the VeritaPolicy approval workflow build as Done (C29),
add #39 MediaLab parity hardening as open follow-on capturing the
60-70% surface assessment and the depth gaps surfaced by the QA pass.

PLAN:
  1. C29 entry: 12 PRs (#438-#449), schema + 8 phases + QA endpoint,
     54/54 happy-path verified.
  2. #39 entry: gaps list (quizzes, watermarking, SSO, delegation,
     etc.) with recommended sequence when customer-triggered.
  3. Re-run scripts/build_parking_lot_xlsx.py per memory rule.

Self-check:
  - Open count drops/rises correctly: was 10, now 11 (added #39).
  - Closed count rises: was 28, now 29 (added C29).
  - No accidental edits to other entries.

Co-authored-by: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1005,8 +1005,56 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>MediaLab parity hardening (VeritaPolicy approval workflow depth)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Open, customer-triggered. No urgency until a prospect specifically asks for one of the listed depth items.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>L (1-2 weeks for the high-value items; each independent feature is M)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Medium-High — the C29 build shipped the surface MediaLab markets but depth is...</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>The VeritaPolicy approval workflow build (C29, 2026-05-29) hit roughly 60-70% MediaLab feature surface. The following gaps remain when comparing against an enterprise MediaLab Document Control deployment:
+- Quizzes on attestations. Schema columns quiz_score and quiz_total_questions exist on policy_attestations but the quiz authoring + presentation UI was scoped out of Phase 4. MediaLab labs use 5-10 multiple-choice questions per policy to confirm comprehension, not just attestation. Adds compliance defensibility.
+- PDF watermarking. MediaLab burns user name + timestamp into every downloaded PDF copy as a deterrent against forwarding. We serve clean originals. Add Puppeteer-style overlay at download time.
+- Per-policy role mapping at department level. MediaLab lets a lab say "only Microbiology Lab Director can approve Microbiology policies." Our required_role is per-step on the workflow, not per-document-by-manual.
+- Approval delegation. When a reviewer is on vacation, MediaLab supports temporary delegation to a designate. We have no delegation model.
+- In-browser DOCX editing. MediaLab has a structured editor that creates a Table of Contents from headings. We treat documents as...</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29 QA pass after C29 shipped (qa-policy-build.js + qa-policy-ui.js: 54/54 happy path verified). Honest depth assessment surfaced by Michael's "how confident are you" question — see C29 entry for full QA receipts.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Post-COLA. Defensive against MediaLab in head-to-head sales calls.
+---</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1017,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2002,8 +2050,44 @@
       </c>
       <c r="H29" s="3" t="inlineStr"/>
     </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>C29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>VeritaPolicy approval workflow — MediaLab functional mirror</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>XL (one focused session, 12 PRs landed)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>High — replaces MediaLab Document Control ($752/$2,250 starting price, scalin...</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Effort: XL (one focused session, 12 PRs landed)
+Importance: High — replaces MediaLab Document Control ($752/$2,250 starting price, scaling to $10K-$20K/yr at enterprise per Capterra public data) with an included VeritaPolicy feature; closes a real positioning gap and gives sales a direct comparator line.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Pricing strategy conversation 2026-05-29 (Michael: "I don't like bolt-ons; we should replicate this") → scoped 8 phases → shipped all 12 PRs in single session. Shipped 2026-05-29.
+---</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H29"/>
+  <autoFilter ref="A1:H30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(parking-lot): revert #40 Longstreth Simple Accuracy entry, renumber Phase A click to #40
TASK: The "Simple Accuracy" toggle ask from Longstreth's 2026-06-02
reply is active work, not parked. Operator clarification: the
parking-lot pass earlier this turn was supposed to park the
in-progress VeritaQC items so we could focus on Longstreth's newest
email, not park Longstreth's ask itself.

PLAN:
  1. Remove the misclassified #40 entry from PARKING_LOT.md.
  2. Renumber the VeritaQC Phase A Gate 3 human click entry from #41
     to #40 so the live-backlog sequence stays contiguous.
  3. Rebuild PARKING_LOT.xlsx via scripts/build_parking_lot_xlsx.py.

Self-check:
  - #40 (Phase A Gate 3 click) is the one genuinely parked item from
    the prior commit; it stays.
  - The Longstreth Simple Accuracy build is now active work and will
    be scoped + authorized in the next round; no parking-lot entry
    needed for active work.
  - Both files committed in lockstep per the xlsx-mirror rule.
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1061,80 +1061,40 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>VeritaCheck Accuracy / Bias module: "Simple Accuracy" vs "Method Comparison" mode toggle (Longstreth ask)</t>
+          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Open, sequencing-dependent. Pre- vs post-COLA: indifferent; this is feature work, not pricing or onboarding.
+          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
 ---</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>M (~half-day: add mode selector to accuracy_bias study type, branch the data-...</t>
+          <t>XS (~5 minutes of Michael's time on a live URL).</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Medium-High. Direct ask from a heavy EP Evaluator user who is otherwise sold...</t>
+          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Effort: M (~half-day: add mode selector to accuracy_bias study type, branch the data-entry form to a Precision-style replicate grid with per-level target value when "Simple Accuracy" is picked, leave existing multi-instrument correlation flow intact for "Method Comparison" mode).
-Importance: Medium-High. Direct ask from a heavy EP Evaluator user who is otherwise sold on the cal_ver split work. Closes the last conceptual friction point for EP-to-Veritas migrators, which Longstreth flagged as "a big selling point" for transition labs.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Longstreth email reply 2026-06-02 (chat parking-lot turn). Build authorization not yet given.</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>VeritaQC Import Phase A: human-in-the-loop Gate 3 click-through (deferred)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Open, awaiting Michael's 5-minute click test. Will move task #77 to completed only after he reports the user-visible result.
----</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>XS (~5 minutes of Michael's time on a live URL).</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Low. Backend contract is fully verified via 35/35 passing offline contract ch...</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Effort: XS (~5 minutes of Michael's time on a live URL).
 Importance: Low. Backend contract is fully verified via 35/35 passing offline contract checks (scripts/verify-veritaqc-import.js) plus three live-API smoke checks against prod (candidates, preview, mappings PUT/GET) on Riverside Regional with seed lot SEED-1780436709094 (18 Glucose results). The browser-driven click was not run because Claude-in-Chrome's renderer froze repeatedly on the Radix Select inside VeritaCheckPage, not on Phase A code itself. Risk of a UX bug surviving to a customer is small but not zero.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>task #77 stalled at Gate 3 step 8 on 2026-06-02. PR #500 squash-merged at commit 17a91ff, prod /api/health confirmed ACTIVE on that commit at 20:43 UTC.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
parking-lot: add entry #42 outbound demo-invite messaging campaign
TASK: Add parking-lot entry #42 documenting the tiered outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts. Deferred from implementation per Michael's request 2026-06-04.

PLAN:
- Write tiered targeting plan (Tier 1 engagers+role through Tier 4 adjacent) to PARKING_LOT.md at end of OPEN section
- Re-run scripts/build_parking_lot_xlsx.py to mirror to PARKING_LOT.xlsx
- Commit both files together per parking-lot auto-sync rule

Self-check:
- Entry numbered #42, next after #41, placed before CLOSED section
- xlsx mirror regenerated, OPEN count now 14 (was 13 before this entry)
- Internal-doc change only, no public-facing copy, Gate 3 N/A
- Committed on feature branch wave-i-3-element5-pt-bridge; entry lands in main when branch merges

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARKING_LOT.xlsx
+++ b/PARKING_LOT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OPEN'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CLOSED'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RETIRED'!$A$1:$H$7</definedName>
   </definedNames>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1133,8 +1133,47 @@
       </c>
       <c r="H14" s="2" t="inlineStr"/>
     </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Outbound demo-invite messaging campaign to 1st-degree LinkedIn contacts</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Parked. Plan documented. Implementation deferred until trigger conditions met.
+---</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>L (1 week prep + 4-6 weeks of staged sends)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>High. Converts existing warm network (~2,500 1st-degree contacts and growing...</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>A staged outbound DM campaign walking Michael's 1st-degree LinkedIn contacts through tier-segmented demo invitations for VeritaAssure. Goal: convert warmest contacts into demo conversations first, then chain into trials and paid subscriptions. Separate pipeline from COLA cohort follow-up and from content-driven inbound; all three feed the same demo funnel but originate from different warmth sources.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 session, after weekly LinkedIn invite batch completion (80 sent, cap hit at #84 Victoria Allen).</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>